<commit_message>
Microsoft Office test files made again from new exports (option B)
the maintainer's 13 saves (Word 16.0, Excel 16.03, PowerPoint 16.0 for Mac) from the packet make.sh
prepared replace the converted ones: hello-table's report, finance and deck re-saves and edits
(and the unlocked report), and the real files' paper, lca-model and milleleaf-deck saves.
Metadata scrubbed as before (last modified by Milleleaf, Excel's folder path trimmed). Every
test file is now as its app saved it; examples/real/SOURCES.md has the new hashes and inputs.

Box: Rust tests 189 passed, 0 failed, 9 ignored; run.sh steps 1-19 exit 0 (step 14: re-saves no
change, Word and Excel edits give the same layers as LibreOffice, PowerPoint 14 matches all
certain; step 18: no PENDING); site build and checks exit 0 (88 PASS).
</commit_message>
<xml_diff>
--- a/examples/hello-table/fixtures/finance.msoffice-edited.xlsx
+++ b/examples/hello-table/fixtures/finance.msoffice-edited.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/examples/hello-table/fixtures/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="~/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A1DB7B9-2ADC-E94A-ACE1-59F570CF0302}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3AA2B976-7664-1349-95FD-DD3469699DF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="34560" windowHeight="22340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Q3 2026" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <definedName name="mleaf_3f1c2a90_0000_4c1e_9a00_000000000011" comment="milleleaf node 3f1c2a90-0000-4c1e-9a00-000000000011">'Q3 2026'!$A$1</definedName>
     <definedName name="mleaf_3f1c2a90_0000_4c1e_9a00_000000000012" comment="milleleaf node 3f1c2a90-0000-4c1e-9a00-000000000012">'Q3 2026'!$A$1:$B$5</definedName>
     <definedName name="mleaf_3f1c2a90_0000_4c1e_9a00_000000000013" comment="milleleaf node 3f1c2a90-0000-4c1e-9a00-000000000013">'Q3 2026'!$B$6</definedName>
-    <definedName name="mleaf_revision">"3b0b95b52b828de91bcdb13f"</definedName>
+    <definedName name="mleaf_revision">"c50ea0fe36a3631b2dbab632"</definedName>
     <definedName name="mleaf_workbook">"3f1c2a90-0000-4c1e-9a00-000000000010"</definedName>
   </definedNames>
   <calcPr calcId="191029"/>

</xml_diff>